<commit_message>
Update FrAppointment PDM et CU PDM 6aea7f03d79528e43e247d8e468acc483ea84a5a
</commit_message>
<xml_diff>
--- a/feature/evolutionRDVV3/ig/StructureDefinition-sas-sos-appointment.xlsx
+++ b/feature/evolutionRDVV3/ig/StructureDefinition-sas-sos-appointment.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-09T15:39:29+00:00</t>
+    <t>2026-09-10T09:13:18+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Profil de Slot, dérivé de FrSlot, pour le service d’agrégation de créneaux de la plateforme SAS - cas d’usage SOS Médecins</t>
+    <t>Profil de Slot, dérivé de FrSlot, pour le service d’agrégation de créneaux de la plateforme SAS - cas d’usage SOS Médecins et Place de Marché</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>